<commit_message>
Fade revenue growth gradually after the consensus window instead of decaying it geometrically
The old path lost ~30% of the excess over the terminal rate every year and, for cyclicals, was capped
at sector growth + 2pp, so growth fell off a cliff right after the consensus years (12% -> 6% in one
year) and sat at trend by year 6. Now:
- linear fade from the last consensus year to the terminal rate (convex for cyclicals)
- cyclical cap relaxed to sector growth + 5pp
- a single consensus year starts the fade 40% of the way back toward sector growth
- the growth exhibit clips year-1 spikes (labelled) so the fade stays readable
- regression test; reports, PDFs, Excel and library regenerated

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Jf4vGSDEJELKK6Wo1Br2bM
</commit_message>
<xml_diff>
--- a/Meridian_demo_report.xlsx
+++ b/Meridian_demo_report.xlsx
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>294.2009389878127</v>
+        <v>298.006665307772</v>
       </c>
     </row>
     <row r="8">
@@ -1355,13 +1355,13 @@
         </is>
       </c>
       <c r="C5" s="6" t="n">
-        <v>230.2679444300176</v>
+        <v>243.0634455376986</v>
       </c>
       <c r="D5" s="6" t="n">
-        <v>195.7932446575796</v>
+        <v>202.3748546056572</v>
       </c>
       <c r="E5" s="6" t="n">
-        <v>270.3739636759826</v>
+        <v>291.6140709499754</v>
       </c>
       <c r="F5" s="11" t="n">
         <v>0.3888888888888889</v>
@@ -1531,7 +1531,7 @@
         </is>
       </c>
       <c r="B18" s="6" t="n">
-        <v>294.2009389878127</v>
+        <v>298.006665307772</v>
       </c>
     </row>
     <row r="20">
@@ -1544,7 +1544,7 @@
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
         <is>
-          <t>Target anchored 30% to the Street consensus ($285.00, 24 analysts); model-only target $298.14.</t>
+          <t>Target anchored 30% to the Street consensus ($285.00, 24 analysts); model-only target $303.58.</t>
         </is>
       </c>
     </row>
@@ -1656,31 +1656,31 @@
         <v>91976.02712078404</v>
       </c>
       <c r="C5" s="18" t="n">
-        <v>97242.50107360962</v>
+        <v>97954.468883635</v>
       </c>
       <c r="D5" s="18" t="n">
-        <v>101922.3637284257</v>
+        <v>103831.7370166531</v>
       </c>
       <c r="E5" s="18" t="n">
-        <v>106160.1062143977</v>
+        <v>109542.482552569</v>
       </c>
       <c r="F5" s="18" t="n">
-        <v>110075.7571630058</v>
+        <v>115019.6066801975</v>
       </c>
       <c r="G5" s="18" t="n">
-        <v>113765.450065953</v>
+        <v>120195.4889808064</v>
       </c>
       <c r="H5" s="18" t="n">
-        <v>117304.4019366943</v>
+        <v>125003.3085400386</v>
       </c>
       <c r="I5" s="18" t="n">
-        <v>120750.5996737408</v>
+        <v>129378.42433894</v>
       </c>
       <c r="J5" s="18" t="n">
-        <v>124148.3572415785</v>
+        <v>133259.7770691082</v>
       </c>
       <c r="K5" s="18" t="n">
-        <v>127252.0661726179</v>
+        <v>136591.2714958359</v>
       </c>
     </row>
     <row r="6">
@@ -1825,31 +1825,31 @@
         <v>20929.320860833</v>
       </c>
       <c r="C9" s="18" t="n">
-        <v>22104.5885545333</v>
+        <v>22269.69061368228</v>
       </c>
       <c r="D9" s="18" t="n">
-        <v>23138.84895703044</v>
+        <v>23580.66883121206</v>
       </c>
       <c r="E9" s="18" t="n">
-        <v>24066.3445679313</v>
+        <v>24847.31857057656</v>
       </c>
       <c r="F9" s="18" t="n">
-        <v>24915.3927733605</v>
+        <v>26054.43047543562</v>
       </c>
       <c r="G9" s="18" t="n">
-        <v>25708.57745523674</v>
+        <v>27186.8095170953</v>
       </c>
       <c r="H9" s="18" t="n">
-        <v>26463.49203784749</v>
+        <v>28229.5793548548</v>
       </c>
       <c r="I9" s="18" t="n">
-        <v>27193.63558442294</v>
+        <v>29168.49630034804</v>
       </c>
       <c r="J9" s="18" t="n">
-        <v>27971.36325082134</v>
+        <v>30056.91618935849</v>
       </c>
       <c r="K9" s="18" t="n">
-        <v>28681.78483209187</v>
+        <v>30819.47659409245</v>
       </c>
     </row>
     <row r="10">
@@ -1909,31 +1909,31 @@
         <v>20305.78018192693</v>
       </c>
       <c r="C12" s="19" t="n">
-        <v>21526.39523626225</v>
+        <v>21576.306040602</v>
       </c>
       <c r="D12" s="19" t="n">
-        <v>22567.06019833192</v>
+        <v>22815.31678354708</v>
       </c>
       <c r="E12" s="19" t="n">
-        <v>23467.17211944108</v>
+        <v>24008.59546516661</v>
       </c>
       <c r="F12" s="19" t="n">
-        <v>24260.42425119743</v>
+        <v>25141.7376855238</v>
       </c>
       <c r="G12" s="19" t="n">
-        <v>24974.21862353873</v>
+        <v>26200.42593427777</v>
       </c>
       <c r="H12" s="19" t="n">
-        <v>25630.12755568923</v>
+        <v>27170.71849549537</v>
       </c>
       <c r="I12" s="19" t="n">
-        <v>26244.76841823402</v>
+        <v>28039.34520228492</v>
       </c>
       <c r="J12" s="19" t="n">
-        <v>26892.84857617929</v>
+        <v>28860.65378038668</v>
       </c>
       <c r="K12" s="19" t="n">
-        <v>27508.67422075087</v>
+        <v>29560.26977075519</v>
       </c>
     </row>
     <row r="13">
@@ -2267,28 +2267,28 @@
         <v>0.07000000000000006</v>
       </c>
       <c r="C26" s="11" t="n">
-        <v>0.05725920239965994</v>
+        <v>0.06500000000000006</v>
       </c>
       <c r="D26" s="11" t="n">
-        <v>0.04812569198804942</v>
+        <v>0.06000000000000005</v>
       </c>
       <c r="E26" s="11" t="n">
-        <v>0.04157814174388176</v>
+        <v>0.05500000000000005</v>
       </c>
       <c r="F26" s="11" t="n">
-        <v>0.03688439177613628</v>
+        <v>0.05000000000000004</v>
       </c>
       <c r="G26" s="11" t="n">
-        <v>0.03351957777118297</v>
+        <v>0.04500000000000003</v>
       </c>
       <c r="H26" s="11" t="n">
-        <v>0.03110743963733855</v>
+        <v>0.04000000000000002</v>
       </c>
       <c r="I26" s="11" t="n">
-        <v>0.02937824736454688</v>
+        <v>0.03500000000000002</v>
       </c>
       <c r="J26" s="11" t="n">
-        <v>0.02813863928641545</v>
+        <v>0.03000000000000001</v>
       </c>
       <c r="K26" s="11" t="n">
         <v>0.025</v>

</xml_diff>